<commit_message>
[BD Log] 18 records — 2026-09-08T23:44
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1099,9 +1099,48 @@
         <v>2026-07-31T04:43:09.254Z</v>
       </c>
     </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19">
+        <v>1788911054554</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="C19" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D19" t="str">
+        <v>08:40</v>
+      </c>
+      <c r="E19" t="str">
+        <v>08:43</v>
+      </c>
+      <c r="F19" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G19">
+        <v>3</v>
+      </c>
+      <c r="H19" t="str">
+        <v>LMS error</v>
+      </c>
+      <c r="I19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lms reset
+BF1.1.15</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v>2026-09-08T23:44:14.554Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 19 records — 2026-09-14T23:17
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1138,9 +1138,47 @@
         <v>2026-09-08T23:44:14.554Z</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20">
+        <v>1789427849533</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="C20" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D20" t="str">
+        <v>08:13</v>
+      </c>
+      <c r="E20" t="str">
+        <v>08:16</v>
+      </c>
+      <c r="F20" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Lms error 1.1.15</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Lms reset</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1789427849533.jpg</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2026-09-14T23:17:29.534Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 20 records — 2026-09-14T23:22
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1176,9 +1176,47 @@
         <v>2026-09-14T23:17:29.534Z</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21">
+        <v>1789428172908</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-09-14</v>
+      </c>
+      <c r="C21" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D21" t="str">
+        <v>08:16</v>
+      </c>
+      <c r="E21" t="str">
+        <v>08:18</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Intralox error wa02.01 850HC intralox 오류</v>
+      </c>
+      <c r="I21" t="str">
+        <v>판넬에서 Reset</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1789428172908.jpg</v>
+      </c>
+      <c r="L21" t="str">
+        <v>2026-09-14T23:22:52.908Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 21 records — 2026-09-15T23:16
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1214,9 +1214,47 @@
         <v>2026-09-14T23:22:52.908Z</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22">
+        <v>1789514189944</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C22" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D22" t="str">
+        <v>08:13</v>
+      </c>
+      <c r="E22" t="str">
+        <v>08:15</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Lms 에러 bf1.1.17</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Lms reset</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1789514189944.jpg</v>
+      </c>
+      <c r="L22" t="str">
+        <v>2026-09-15T23:16:29.944Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 22 records — 2026-09-15T23:31
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1252,9 +1252,47 @@
         <v>2026-09-15T23:16:29.944Z</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23">
+        <v>1789515084765</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C23" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D23" t="str">
+        <v>08:29</v>
+      </c>
+      <c r="E23" t="str">
+        <v>08:31</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Lms error 1.1.15</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Lms reset</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v>2026-09-15T23:31:24.765Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 23 records — 2026-09-15T23:44
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1290,9 +1290,47 @@
         <v>2026-09-15T23:31:24.765Z</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24">
+        <v>1789515858141</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C24" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D24" t="str">
+        <v>08:43</v>
+      </c>
+      <c r="E24" t="str">
+        <v>08:45</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Lms 1.1.11 error</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Error reset</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v>2026-09-15T23:44:18.141Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 24 records — 2026-09-15T23:59
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1328,9 +1328,47 @@
         <v>2026-09-15T23:44:18.141Z</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25">
+        <v>1789516770614</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="C25" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D25" t="str">
+        <v>08:57</v>
+      </c>
+      <c r="E25" t="str">
+        <v>08:59</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Lms 1.1.11 error</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Reset</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v>2026-09-15T23:59:30.614Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 25 records — 2026-09-16T23:03
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1366,9 +1366,47 @@
         <v>2026-09-15T23:59:30.614Z</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26">
+        <v>1789599797477</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C26" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D26" t="str">
+        <v>08:00</v>
+      </c>
+      <c r="E26" t="str">
+        <v>08:02</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2분</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Lms error 1.1.15</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Reset</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v>2026-09-16T23:03:17.477Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 26 records — 2026-09-17T00:21
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1404,9 +1404,47 @@
         <v>2026-09-16T23:03:17.477Z</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27">
+        <v>1789604503126</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C27" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D27" t="str">
+        <v>08:50</v>
+      </c>
+      <c r="E27" t="str">
+        <v>09:15</v>
+      </c>
+      <c r="F27" t="str">
+        <v>25분</v>
+      </c>
+      <c r="G27">
+        <v>25</v>
+      </c>
+      <c r="H27" t="str">
+        <v>WE02.02.046sf 파워롤러(L885)선 꼬임</v>
+      </c>
+      <c r="I27" t="str">
+        <v>전원선 복구 재설치</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v>2026-09-17T00:21:43.126Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>